<commit_message>
corrections according to List
corrections according to lists (person, place, org) finished
</commit_message>
<xml_diff>
--- a/data/xlsx/Baernreither_Ortsregister_2023.xlsx
+++ b/data/xlsx/Baernreither_Ortsregister_2023.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/christofaichner/Documents/GitHub/baernreither-data/data/xlsx/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E8732C83-ADF7-854F-9F06-7EAC4B0BE8B0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{985F91BC-B6BE-0D47-9371-6B63A431C740}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="760" windowWidth="29400" windowHeight="16440" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -3976,7 +3976,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="35" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="89">
+  <cellXfs count="87">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -4188,10 +4188,6 @@
     <xf numFmtId="0" fontId="35" fillId="3" borderId="0" xfId="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="39" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="35" fillId="2" borderId="0" xfId="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
@@ -4526,16 +4522,16 @@
       </c>
     </row>
     <row r="4" spans="1:25" ht="16">
-      <c r="A4" s="81" t="s">
+      <c r="A4" s="3" t="s">
         <v>1051</v>
       </c>
-      <c r="B4" s="81" t="s">
+      <c r="B4" s="3" t="s">
         <v>1052</v>
       </c>
-      <c r="C4" s="81" t="s">
+      <c r="C4" s="3" t="s">
         <v>1053</v>
       </c>
-      <c r="D4" s="82" t="s">
+      <c r="D4" s="1" t="s">
         <v>1051</v>
       </c>
     </row>
@@ -5684,7 +5680,7 @@
         <v>1036</v>
       </c>
       <c r="B39" s="3"/>
-      <c r="C39" s="3" t="s">
+      <c r="C39" s="50" t="s">
         <v>1037</v>
       </c>
       <c r="D39" s="1" t="s">
@@ -6092,7 +6088,7 @@
         <v>935</v>
       </c>
       <c r="B51" s="3"/>
-      <c r="C51" s="3" t="s">
+      <c r="C51" s="50" t="s">
         <v>936</v>
       </c>
       <c r="D51" s="1" t="s">
@@ -10026,13 +10022,13 @@
       <c r="Y166" s="1"/>
     </row>
     <row r="167" spans="1:25" ht="15" customHeight="1">
-      <c r="A167" s="83" t="s">
+      <c r="A167" s="81" t="s">
         <v>1096</v>
       </c>
       <c r="C167" t="s">
         <v>1097</v>
       </c>
-      <c r="D167" s="83" t="s">
+      <c r="D167" s="81" t="s">
         <v>1096</v>
       </c>
     </row>
@@ -10696,7 +10692,7 @@
       <c r="B187" s="5" t="s">
         <v>1103</v>
       </c>
-      <c r="C187" s="84" t="s">
+      <c r="C187" s="82" t="s">
         <v>1104</v>
       </c>
       <c r="D187" s="5" t="s">
@@ -10731,7 +10727,7 @@
       <c r="B188" s="5" t="s">
         <v>1105</v>
       </c>
-      <c r="C188" s="84" t="s">
+      <c r="C188" s="82" t="s">
         <v>1106</v>
       </c>
       <c r="D188" s="5" t="s">
@@ -13513,7 +13509,7 @@
       <c r="Y269" s="2"/>
     </row>
     <row r="270" spans="1:25" ht="15.75" customHeight="1">
-      <c r="A270" s="85" t="s">
+      <c r="A270" s="83" t="s">
         <v>1128</v>
       </c>
       <c r="B270" s="7"/>
@@ -16066,7 +16062,7 @@
       <c r="Y344" s="1"/>
     </row>
     <row r="345" spans="1:25" ht="15.75" customHeight="1">
-      <c r="A345" s="83" t="s">
+      <c r="A345" s="81" t="s">
         <v>1140</v>
       </c>
       <c r="B345" s="13" t="s">
@@ -16101,16 +16097,16 @@
       <c r="Y345" s="1"/>
     </row>
     <row r="346" spans="1:25" ht="15.75" customHeight="1">
-      <c r="A346" s="86" t="s">
+      <c r="A346" s="84" t="s">
         <v>1143</v>
       </c>
-      <c r="B346" s="87" t="s">
+      <c r="B346" s="85" t="s">
         <v>1142</v>
       </c>
-      <c r="C346" s="88" t="s">
+      <c r="C346" s="86" t="s">
         <v>1144</v>
       </c>
-      <c r="D346" s="87" t="s">
+      <c r="D346" s="85" t="s">
         <v>1143</v>
       </c>
       <c r="E346" s="1"/>
@@ -23664,11 +23660,13 @@
     <hyperlink ref="C187" r:id="rId263" xr:uid="{3DD3F81F-9B00-6C41-B9BD-0B246E4511FC}"/>
     <hyperlink ref="C246" r:id="rId264" xr:uid="{2653430D-3B53-3342-82F4-5C182DA7B834}"/>
     <hyperlink ref="C143" r:id="rId265" xr:uid="{A86712C1-CF60-EC43-ACC0-2F9F008D6A13}"/>
+    <hyperlink ref="C39" r:id="rId266" xr:uid="{DEDBA11F-1236-FB46-9BF5-3341C3B4F82F}"/>
+    <hyperlink ref="C51" r:id="rId267" xr:uid="{A2CD9817-DB83-EB44-B2B9-3529BB5D6BE5}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0" footer="0"/>
   <pageSetup paperSize="9" orientation="portrait"/>
   <tableParts count="1">
-    <tablePart r:id="rId266"/>
+    <tablePart r:id="rId268"/>
   </tableParts>
 </worksheet>
 </file>

</xml_diff>